<commit_message>
Update data model Excel to document planned DIM_DATE table
Adds DimDate as a planned (not yet implemented) addition across all sheets
in green — fields, constraints, relationships, and a step-by-step implementation
plan sheet. Existing current-state rows are unchanged.

https://claude.ai/code/session_01FWDc8DouqVfP9aMm2wroty
</commit_message>
<xml_diff>
--- a/budget_data_model.xlsx
+++ b/budget_data_model.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Constraints &amp; Indexes" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Relationships" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Business Logic" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="DimDate Plan" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -57,8 +58,20 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00375623"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00375623"/>
+      <sz val="14"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -85,8 +98,23 @@
         <fgColor rgb="002E75B6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00375623"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -100,11 +128,39 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -123,6 +179,29 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -489,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -951,10 +1030,55 @@
       </c>
       <c r="G14" s="4" t="inlineStr"/>
     </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↓  PLANNED ADDITIONS  (not yet implemented — green rows)  ↓</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="60" customHeight="1">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>dim_date_dimdate</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>dim_date (new app)</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Date dimension: one row per calendar day 2000-01-01→2039-12-31. All date FK fields will reference this table.</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>date (PK), year, month, day, quarter, day_of_week, day_of_year, week_of_year, is_weekday, is_weekend, day_name, month_name, month_abbrev, year_month, days_in_month, is_month_start, is_month_end, month_start_date, month_end_date, is_quarter_start, is_quarter_end, quarter_start_date, quarter_end_date, is_year_start, is_year_end</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>No FK parents (standalone lookup table). Will be referenced by: Budget.month, GoalAllocation.month, JournalEntry.entry_date, and other DateFields.</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>date is the PK (DateField). No team scoping — global shared table. Populated via manage.py populate_dim_date.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A15:G15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -966,7 +1090,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I96"/>
+  <dimension ref="A1:I122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1033,6 +1157,14 @@
           <t xml:space="preserve">  BaseModel (abstract)</t>
         </is>
       </c>
+      <c r="B2" s="9" t="n"/>
+      <c r="C2" s="9" t="n"/>
+      <c r="D2" s="9" t="n"/>
+      <c r="E2" s="9" t="n"/>
+      <c r="F2" s="9" t="n"/>
+      <c r="G2" s="9" t="n"/>
+      <c r="H2" s="9" t="n"/>
+      <c r="I2" s="10" t="n"/>
     </row>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
@@ -1196,6 +1328,14 @@
           <t xml:space="preserve">  Budget</t>
         </is>
       </c>
+      <c r="B7" s="9" t="n"/>
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="9" t="n"/>
+      <c r="G7" s="9" t="n"/>
+      <c r="H7" s="9" t="n"/>
+      <c r="I7" s="10" t="n"/>
     </row>
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
@@ -1578,6 +1718,14 @@
           <t xml:space="preserve">  Goal</t>
         </is>
       </c>
+      <c r="B17" s="9" t="n"/>
+      <c r="C17" s="9" t="n"/>
+      <c r="D17" s="9" t="n"/>
+      <c r="E17" s="9" t="n"/>
+      <c r="F17" s="9" t="n"/>
+      <c r="G17" s="9" t="n"/>
+      <c r="H17" s="9" t="n"/>
+      <c r="I17" s="10" t="n"/>
     </row>
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
@@ -2116,6 +2264,14 @@
           <t xml:space="preserve">  GoalAllocation</t>
         </is>
       </c>
+      <c r="B31" s="9" t="n"/>
+      <c r="C31" s="9" t="n"/>
+      <c r="D31" s="9" t="n"/>
+      <c r="E31" s="9" t="n"/>
+      <c r="F31" s="9" t="n"/>
+      <c r="G31" s="9" t="n"/>
+      <c r="H31" s="9" t="n"/>
+      <c r="I31" s="10" t="n"/>
     </row>
     <row r="32" ht="16" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
@@ -2533,6 +2689,14 @@
           <t xml:space="preserve">  AccountGroup</t>
         </is>
       </c>
+      <c r="B42" s="9" t="n"/>
+      <c r="C42" s="9" t="n"/>
+      <c r="D42" s="9" t="n"/>
+      <c r="E42" s="9" t="n"/>
+      <c r="F42" s="9" t="n"/>
+      <c r="G42" s="9" t="n"/>
+      <c r="H42" s="9" t="n"/>
+      <c r="I42" s="10" t="n"/>
     </row>
     <row r="43" ht="16" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
@@ -2903,6 +3067,14 @@
           <t xml:space="preserve">  Account</t>
         </is>
       </c>
+      <c r="B52" s="9" t="n"/>
+      <c r="C52" s="9" t="n"/>
+      <c r="D52" s="9" t="n"/>
+      <c r="E52" s="9" t="n"/>
+      <c r="F52" s="9" t="n"/>
+      <c r="G52" s="9" t="n"/>
+      <c r="H52" s="9" t="n"/>
+      <c r="I52" s="10" t="n"/>
     </row>
     <row r="53" ht="16" customHeight="1">
       <c r="A53" s="4" t="inlineStr">
@@ -3328,6 +3500,14 @@
           <t xml:space="preserve">  Payee</t>
         </is>
       </c>
+      <c r="B63" s="9" t="n"/>
+      <c r="C63" s="9" t="n"/>
+      <c r="D63" s="9" t="n"/>
+      <c r="E63" s="9" t="n"/>
+      <c r="F63" s="9" t="n"/>
+      <c r="G63" s="9" t="n"/>
+      <c r="H63" s="9" t="n"/>
+      <c r="I63" s="10" t="n"/>
     </row>
     <row r="64" ht="16" customHeight="1">
       <c r="A64" s="4" t="inlineStr">
@@ -3624,6 +3804,14 @@
           <t xml:space="preserve">  JournalEntry</t>
         </is>
       </c>
+      <c r="B71" s="9" t="n"/>
+      <c r="C71" s="9" t="n"/>
+      <c r="D71" s="9" t="n"/>
+      <c r="E71" s="9" t="n"/>
+      <c r="F71" s="9" t="n"/>
+      <c r="G71" s="9" t="n"/>
+      <c r="H71" s="9" t="n"/>
+      <c r="I71" s="10" t="n"/>
     </row>
     <row r="72" ht="16" customHeight="1">
       <c r="A72" s="4" t="inlineStr">
@@ -4084,6 +4272,14 @@
           <t xml:space="preserve">  JournalLine</t>
         </is>
       </c>
+      <c r="B83" s="9" t="n"/>
+      <c r="C83" s="9" t="n"/>
+      <c r="D83" s="9" t="n"/>
+      <c r="E83" s="9" t="n"/>
+      <c r="F83" s="9" t="n"/>
+      <c r="G83" s="9" t="n"/>
+      <c r="H83" s="9" t="n"/>
+      <c r="I83" s="10" t="n"/>
     </row>
     <row r="84" ht="16" customHeight="1">
       <c r="A84" s="4" t="inlineStr">
@@ -4636,8 +4832,990 @@
         </is>
       </c>
     </row>
+    <row r="97" ht="18" customHeight="1">
+      <c r="A97" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  DimDate  [PLANNED — new app: apps/dim_date]</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="16" customHeight="1">
+      <c r="A98" s="8" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B98" s="8" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="C98" s="8" t="inlineStr">
+        <is>
+          <t>DateField (PK)</t>
+        </is>
+      </c>
+      <c r="D98" s="8" t="inlineStr">
+        <is>
+          <t>date PK</t>
+        </is>
+      </c>
+      <c r="E98" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F98" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G98" s="8" t="inlineStr"/>
+      <c r="H98" s="8" t="inlineStr">
+        <is>
+          <t>PRIMARY KEY</t>
+        </is>
+      </c>
+      <c r="I98" s="8" t="inlineStr">
+        <is>
+          <t>Natural key; FK target for all date fields</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="16" customHeight="1">
+      <c r="A99" s="12" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B99" s="12" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="C99" s="12" t="inlineStr">
+        <is>
+          <t>SmallIntegerField</t>
+        </is>
+      </c>
+      <c r="D99" s="12" t="inlineStr">
+        <is>
+          <t>smallint</t>
+        </is>
+      </c>
+      <c r="E99" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F99" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G99" s="12" t="inlineStr"/>
+      <c r="H99" s="12" t="inlineStr"/>
+      <c r="I99" s="12" t="inlineStr"/>
+    </row>
+    <row r="100" ht="16" customHeight="1">
+      <c r="A100" s="8" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B100" s="8" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="C100" s="8" t="inlineStr">
+        <is>
+          <t>SmallIntegerField</t>
+        </is>
+      </c>
+      <c r="D100" s="8" t="inlineStr">
+        <is>
+          <t>smallint</t>
+        </is>
+      </c>
+      <c r="E100" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F100" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G100" s="8" t="inlineStr"/>
+      <c r="H100" s="8" t="inlineStr">
+        <is>
+          <t>1–12</t>
+        </is>
+      </c>
+      <c r="I100" s="8" t="inlineStr"/>
+    </row>
+    <row r="101" ht="16" customHeight="1">
+      <c r="A101" s="12" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B101" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="C101" s="12" t="inlineStr">
+        <is>
+          <t>SmallIntegerField</t>
+        </is>
+      </c>
+      <c r="D101" s="12" t="inlineStr">
+        <is>
+          <t>smallint</t>
+        </is>
+      </c>
+      <c r="E101" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F101" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G101" s="12" t="inlineStr"/>
+      <c r="H101" s="12" t="inlineStr">
+        <is>
+          <t>1–31</t>
+        </is>
+      </c>
+      <c r="I101" s="12" t="inlineStr"/>
+    </row>
+    <row r="102" ht="16" customHeight="1">
+      <c r="A102" s="8" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B102" s="8" t="inlineStr">
+        <is>
+          <t>quarter</t>
+        </is>
+      </c>
+      <c r="C102" s="8" t="inlineStr">
+        <is>
+          <t>SmallIntegerField</t>
+        </is>
+      </c>
+      <c r="D102" s="8" t="inlineStr">
+        <is>
+          <t>smallint</t>
+        </is>
+      </c>
+      <c r="E102" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F102" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G102" s="8" t="inlineStr"/>
+      <c r="H102" s="8" t="inlineStr">
+        <is>
+          <t>1–4</t>
+        </is>
+      </c>
+      <c r="I102" s="8" t="inlineStr"/>
+    </row>
+    <row r="103" ht="16" customHeight="1">
+      <c r="A103" s="12" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B103" s="12" t="inlineStr">
+        <is>
+          <t>day_of_week</t>
+        </is>
+      </c>
+      <c r="C103" s="12" t="inlineStr">
+        <is>
+          <t>SmallIntegerField</t>
+        </is>
+      </c>
+      <c r="D103" s="12" t="inlineStr">
+        <is>
+          <t>smallint</t>
+        </is>
+      </c>
+      <c r="E103" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F103" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G103" s="12" t="inlineStr"/>
+      <c r="H103" s="12" t="inlineStr">
+        <is>
+          <t>ISO: 1=Mon … 7=Sun</t>
+        </is>
+      </c>
+      <c r="I103" s="12" t="inlineStr"/>
+    </row>
+    <row r="104" ht="16" customHeight="1">
+      <c r="A104" s="8" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B104" s="8" t="inlineStr">
+        <is>
+          <t>day_of_year</t>
+        </is>
+      </c>
+      <c r="C104" s="8" t="inlineStr">
+        <is>
+          <t>SmallIntegerField</t>
+        </is>
+      </c>
+      <c r="D104" s="8" t="inlineStr">
+        <is>
+          <t>smallint</t>
+        </is>
+      </c>
+      <c r="E104" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F104" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G104" s="8" t="inlineStr"/>
+      <c r="H104" s="8" t="inlineStr">
+        <is>
+          <t>1–366</t>
+        </is>
+      </c>
+      <c r="I104" s="8" t="inlineStr"/>
+    </row>
+    <row r="105" ht="16" customHeight="1">
+      <c r="A105" s="12" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B105" s="12" t="inlineStr">
+        <is>
+          <t>week_of_year</t>
+        </is>
+      </c>
+      <c r="C105" s="12" t="inlineStr">
+        <is>
+          <t>SmallIntegerField</t>
+        </is>
+      </c>
+      <c r="D105" s="12" t="inlineStr">
+        <is>
+          <t>smallint</t>
+        </is>
+      </c>
+      <c r="E105" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F105" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G105" s="12" t="inlineStr"/>
+      <c r="H105" s="12" t="inlineStr">
+        <is>
+          <t>ISO week 1–53</t>
+        </is>
+      </c>
+      <c r="I105" s="12" t="inlineStr"/>
+    </row>
+    <row r="106" ht="16" customHeight="1">
+      <c r="A106" s="8" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B106" s="8" t="inlineStr">
+        <is>
+          <t>is_weekday</t>
+        </is>
+      </c>
+      <c r="C106" s="8" t="inlineStr">
+        <is>
+          <t>BooleanField</t>
+        </is>
+      </c>
+      <c r="D106" s="8" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="E106" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F106" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G106" s="8" t="inlineStr"/>
+      <c r="H106" s="8" t="inlineStr"/>
+      <c r="I106" s="8" t="inlineStr">
+        <is>
+          <t>True Mon–Fri</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="16" customHeight="1">
+      <c r="A107" s="12" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B107" s="12" t="inlineStr">
+        <is>
+          <t>is_weekend</t>
+        </is>
+      </c>
+      <c r="C107" s="12" t="inlineStr">
+        <is>
+          <t>BooleanField</t>
+        </is>
+      </c>
+      <c r="D107" s="12" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="E107" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F107" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G107" s="12" t="inlineStr"/>
+      <c r="H107" s="12" t="inlineStr"/>
+      <c r="I107" s="12" t="inlineStr">
+        <is>
+          <t>True Sat–Sun</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="16" customHeight="1">
+      <c r="A108" s="8" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B108" s="8" t="inlineStr">
+        <is>
+          <t>day_name</t>
+        </is>
+      </c>
+      <c r="C108" s="8" t="inlineStr">
+        <is>
+          <t>CharField</t>
+        </is>
+      </c>
+      <c r="D108" s="8" t="inlineStr">
+        <is>
+          <t>varchar(9)</t>
+        </is>
+      </c>
+      <c r="E108" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F108" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G108" s="8" t="inlineStr"/>
+      <c r="H108" s="8" t="inlineStr">
+        <is>
+          <t>max_length=9</t>
+        </is>
+      </c>
+      <c r="I108" s="8" t="inlineStr">
+        <is>
+          <t>e.g. Monday</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="16" customHeight="1">
+      <c r="A109" s="12" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B109" s="12" t="inlineStr">
+        <is>
+          <t>month_name</t>
+        </is>
+      </c>
+      <c r="C109" s="12" t="inlineStr">
+        <is>
+          <t>CharField</t>
+        </is>
+      </c>
+      <c r="D109" s="12" t="inlineStr">
+        <is>
+          <t>varchar(9)</t>
+        </is>
+      </c>
+      <c r="E109" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F109" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G109" s="12" t="inlineStr"/>
+      <c r="H109" s="12" t="inlineStr">
+        <is>
+          <t>max_length=9</t>
+        </is>
+      </c>
+      <c r="I109" s="12" t="inlineStr">
+        <is>
+          <t>e.g. January</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="16" customHeight="1">
+      <c r="A110" s="8" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B110" s="8" t="inlineStr">
+        <is>
+          <t>month_abbrev</t>
+        </is>
+      </c>
+      <c r="C110" s="8" t="inlineStr">
+        <is>
+          <t>CharField</t>
+        </is>
+      </c>
+      <c r="D110" s="8" t="inlineStr">
+        <is>
+          <t>varchar(3)</t>
+        </is>
+      </c>
+      <c r="E110" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F110" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G110" s="8" t="inlineStr"/>
+      <c r="H110" s="8" t="inlineStr">
+        <is>
+          <t>max_length=3</t>
+        </is>
+      </c>
+      <c r="I110" s="8" t="inlineStr">
+        <is>
+          <t>e.g. Jan</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="16" customHeight="1">
+      <c r="A111" s="12" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B111" s="12" t="inlineStr">
+        <is>
+          <t>year_month</t>
+        </is>
+      </c>
+      <c r="C111" s="12" t="inlineStr">
+        <is>
+          <t>CharField</t>
+        </is>
+      </c>
+      <c r="D111" s="12" t="inlineStr">
+        <is>
+          <t>varchar(7)</t>
+        </is>
+      </c>
+      <c r="E111" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F111" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G111" s="12" t="inlineStr"/>
+      <c r="H111" s="12" t="inlineStr">
+        <is>
+          <t>max_length=7</t>
+        </is>
+      </c>
+      <c r="I111" s="12" t="inlineStr">
+        <is>
+          <t>YYYY-MM; indexed</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="16" customHeight="1">
+      <c r="A112" s="8" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B112" s="8" t="inlineStr">
+        <is>
+          <t>days_in_month</t>
+        </is>
+      </c>
+      <c r="C112" s="8" t="inlineStr">
+        <is>
+          <t>SmallIntegerField</t>
+        </is>
+      </c>
+      <c r="D112" s="8" t="inlineStr">
+        <is>
+          <t>smallint</t>
+        </is>
+      </c>
+      <c r="E112" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F112" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G112" s="8" t="inlineStr"/>
+      <c r="H112" s="8" t="inlineStr">
+        <is>
+          <t>28–31</t>
+        </is>
+      </c>
+      <c r="I112" s="8" t="inlineStr"/>
+    </row>
+    <row r="113" ht="16" customHeight="1">
+      <c r="A113" s="12" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B113" s="12" t="inlineStr">
+        <is>
+          <t>is_month_start</t>
+        </is>
+      </c>
+      <c r="C113" s="12" t="inlineStr">
+        <is>
+          <t>BooleanField</t>
+        </is>
+      </c>
+      <c r="D113" s="12" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="E113" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F113" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G113" s="12" t="inlineStr"/>
+      <c r="H113" s="12" t="inlineStr"/>
+      <c r="I113" s="12" t="inlineStr">
+        <is>
+          <t>True on the 1st</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="16" customHeight="1">
+      <c r="A114" s="8" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B114" s="8" t="inlineStr">
+        <is>
+          <t>is_month_end</t>
+        </is>
+      </c>
+      <c r="C114" s="8" t="inlineStr">
+        <is>
+          <t>BooleanField</t>
+        </is>
+      </c>
+      <c r="D114" s="8" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="E114" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F114" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G114" s="8" t="inlineStr"/>
+      <c r="H114" s="8" t="inlineStr"/>
+      <c r="I114" s="8" t="inlineStr">
+        <is>
+          <t>True on last day of month</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="16" customHeight="1">
+      <c r="A115" s="12" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B115" s="12" t="inlineStr">
+        <is>
+          <t>month_start_date</t>
+        </is>
+      </c>
+      <c r="C115" s="12" t="inlineStr">
+        <is>
+          <t>DateField</t>
+        </is>
+      </c>
+      <c r="D115" s="12" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="E115" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F115" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G115" s="12" t="inlineStr"/>
+      <c r="H115" s="12" t="inlineStr"/>
+      <c r="I115" s="12" t="inlineStr">
+        <is>
+          <t>First day of this date's month</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="16" customHeight="1">
+      <c r="A116" s="8" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B116" s="8" t="inlineStr">
+        <is>
+          <t>month_end_date</t>
+        </is>
+      </c>
+      <c r="C116" s="8" t="inlineStr">
+        <is>
+          <t>DateField</t>
+        </is>
+      </c>
+      <c r="D116" s="8" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="E116" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F116" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G116" s="8" t="inlineStr"/>
+      <c r="H116" s="8" t="inlineStr"/>
+      <c r="I116" s="8" t="inlineStr">
+        <is>
+          <t>Last day of this date's month</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="16" customHeight="1">
+      <c r="A117" s="12" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B117" s="12" t="inlineStr">
+        <is>
+          <t>is_quarter_start</t>
+        </is>
+      </c>
+      <c r="C117" s="12" t="inlineStr">
+        <is>
+          <t>BooleanField</t>
+        </is>
+      </c>
+      <c r="D117" s="12" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="E117" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F117" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G117" s="12" t="inlineStr"/>
+      <c r="H117" s="12" t="inlineStr"/>
+      <c r="I117" s="12" t="inlineStr"/>
+    </row>
+    <row r="118" ht="16" customHeight="1">
+      <c r="A118" s="8" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B118" s="8" t="inlineStr">
+        <is>
+          <t>is_quarter_end</t>
+        </is>
+      </c>
+      <c r="C118" s="8" t="inlineStr">
+        <is>
+          <t>BooleanField</t>
+        </is>
+      </c>
+      <c r="D118" s="8" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="E118" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F118" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G118" s="8" t="inlineStr"/>
+      <c r="H118" s="8" t="inlineStr"/>
+      <c r="I118" s="8" t="inlineStr"/>
+    </row>
+    <row r="119" ht="16" customHeight="1">
+      <c r="A119" s="12" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B119" s="12" t="inlineStr">
+        <is>
+          <t>quarter_start_date</t>
+        </is>
+      </c>
+      <c r="C119" s="12" t="inlineStr">
+        <is>
+          <t>DateField</t>
+        </is>
+      </c>
+      <c r="D119" s="12" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="E119" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F119" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G119" s="12" t="inlineStr"/>
+      <c r="H119" s="12" t="inlineStr"/>
+      <c r="I119" s="12" t="inlineStr"/>
+    </row>
+    <row r="120" ht="16" customHeight="1">
+      <c r="A120" s="8" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B120" s="8" t="inlineStr">
+        <is>
+          <t>quarter_end_date</t>
+        </is>
+      </c>
+      <c r="C120" s="8" t="inlineStr">
+        <is>
+          <t>DateField</t>
+        </is>
+      </c>
+      <c r="D120" s="8" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="E120" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F120" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G120" s="8" t="inlineStr"/>
+      <c r="H120" s="8" t="inlineStr"/>
+      <c r="I120" s="8" t="inlineStr"/>
+    </row>
+    <row r="121" ht="16" customHeight="1">
+      <c r="A121" s="12" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B121" s="12" t="inlineStr">
+        <is>
+          <t>is_year_start</t>
+        </is>
+      </c>
+      <c r="C121" s="12" t="inlineStr">
+        <is>
+          <t>BooleanField</t>
+        </is>
+      </c>
+      <c r="D121" s="12" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="E121" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F121" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G121" s="12" t="inlineStr"/>
+      <c r="H121" s="12" t="inlineStr"/>
+      <c r="I121" s="12" t="inlineStr">
+        <is>
+          <t>True on Jan 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="16" customHeight="1">
+      <c r="A122" s="8" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B122" s="8" t="inlineStr">
+        <is>
+          <t>is_year_end</t>
+        </is>
+      </c>
+      <c r="C122" s="8" t="inlineStr">
+        <is>
+          <t>BooleanField</t>
+        </is>
+      </c>
+      <c r="D122" s="8" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="E122" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F122" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G122" s="8" t="inlineStr"/>
+      <c r="H122" s="8" t="inlineStr"/>
+      <c r="I122" s="8" t="inlineStr">
+        <is>
+          <t>True on Dec 31</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="A52:I52"/>
     <mergeCell ref="A7:I7"/>
     <mergeCell ref="A2:I2"/>
@@ -4646,6 +5824,7 @@
     <mergeCell ref="A42:I42"/>
     <mergeCell ref="A17:I17"/>
     <mergeCell ref="A31:I31"/>
+    <mergeCell ref="A97:I97"/>
     <mergeCell ref="A83:I83"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4658,7 +5837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5126,7 +6305,167 @@
         </is>
       </c>
     </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  DimDate  [PLANNED]</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>dim_date_dimdate</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>PRIMARY KEY</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>Natural key; no surrogate ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>dim_date_dimdate</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>INDEX</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>year, month</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>dim_date_dimdate</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>INDEX</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>year, quarter</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>dim_date_dimdate</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>INDEX</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>year_month</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>dim_date_dimdate</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>ORDER BY</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>Default queryset ordering</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>dim_date_dimdate</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>DATA RANGE</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>2000-01-01 → 2039-12-31</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>14,610 rows total; populated via populate_dim_date mgmt command</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A19:E19"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5137,7 +6476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5841,7 +7180,165 @@
       </c>
       <c r="G20" s="4" t="inlineStr"/>
     </row>
+    <row r="21" ht="16" customHeight="1">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Planned FK changes — existing DateFields → DimDate  [PLANNED]</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Budget</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>FK (N→1) [planned]</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>PROTECT</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>Replaces plain DateField</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>GoalAllocation</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>FK (N→1) [planned]</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="inlineStr">
+        <is>
+          <t>PROTECT</t>
+        </is>
+      </c>
+      <c r="F23" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G23" s="12" t="inlineStr">
+        <is>
+          <t>Replaces plain DateField</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>JournalEntry</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>entry_date</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>FK (N→1) [planned]</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>PROTECT</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>Replaces plain DateField</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>GoalAllocation</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>month (normalise hook)</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>DimDate</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F25" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G25" s="12" t="inlineStr">
+        <is>
+          <t>Month-normalise-to-1st logic must still run before FK lookup</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A21:G21"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6251,4 +7748,353 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>DIM_DATE — Implementation Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Status: PLANNED (not yet implemented)  |  Green rows in other sheets show the intended changes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>File / Location</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Detail</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Impact</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="55" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>Create new Django app</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>apps/dim_date/</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>New app: apps.py (DimDateConfig), models.py (DimDate), migrations/0001_initial.py</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>None — no existing code touched</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>App needs adding to PROJECT_APPS in settings.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="55" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>Register app in settings</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>koala_budget/settings.py → PROJECT_APPS</t>
+        </is>
+      </c>
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>Add "apps.dim_date.apps.DimDateConfig"</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F5" s="15" t="inlineStr"/>
+    </row>
+    <row r="6" ht="55" customHeight="1">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>Run migration</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>python manage.py migrate dim_date</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>Creates dim_date_dimdate table in DB</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>14,610 rows will be empty until step 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="55" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>Populate table</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>python manage.py populate_dim_date</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>Inserts 14,610 rows (2000-01-01 → 2039-12-31) in batches of 1000</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>Idempotent; --replace flag to rebuild from scratch</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="55" customHeight="1">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>Migrate Budget.month → FK</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>apps/budget/models.py + new migration</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>Change month=DateField() to month=ForeignKey('dim_date.DimDate', …)
+Migration: AddField + data migration to backfill + AlterField + RemoveOld</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>All Budget queries that filter/annotate by month must use month_id (the date value) — existing code mostly unchanged since FK value = date string</t>
+        </is>
+      </c>
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>BudgetService.available() rollover logic uses month arithmetic — review carefully</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="55" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>Migrate GoalAllocation.month → FK</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>apps/budget/models.py + new migration</t>
+        </is>
+      </c>
+      <c r="D9" s="15" t="inlineStr">
+        <is>
+          <t>Same pattern as step 5. Keep month-normalise-to-1st logic in save().</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>GoalService and GoalQuerySet.with_progress() filter by month — verify no breakage</t>
+        </is>
+      </c>
+      <c r="F9" s="15" t="inlineStr"/>
+    </row>
+    <row r="10" ht="55" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>Migrate JournalEntry.entry_date → FK</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>apps/journal/models.py + new migration</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>Change entry_date=DateField() to FK. JournalLine._calculate_budget() derives month from entry_date — must use entry_date_id.replace(day=1) after the change.</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>High impact: JournalEntry is central. All views/serializers referencing entry_date need review.</t>
+        </is>
+      </c>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t>Consider doing in a separate PR</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="55" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>Update admin / serializers / templates</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>Various</t>
+        </is>
+      </c>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>Any admin list_display, serializer fields, or template tags using the migrated date fields may need updating (ForeignKey vs DateField rendering differs).</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>UI/cosmetic; no data loss</t>
+        </is>
+      </c>
+      <c r="F11" s="15" t="inlineStr"/>
+    </row>
+    <row r="12" ht="55" customHeight="1">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>Add populate_dim_date to deployment runbook</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>CI / deployment docs</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>Run manage.py populate_dim_date once per environment after migration.</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="inlineStr">
+        <is>
+          <t>None if forgotten — FK inserts will fail until table is populated</t>
+        </is>
+      </c>
+      <c r="F12" s="14" t="inlineStr">
+        <is>
+          <t>Consider adding to post-migrate signal or fixture</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>